<commit_message>
Lambda OMS 2023-10-19 销售订单 迭代开发bug 修复
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/PIDomestic.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/PIDomestic.xlsx
@@ -363,13 +363,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">MIC CO.,LTD
-3-408 SUZUKI-CHO 1-72-1 KODAIRA-SHI, TOKYO 187-0011 JAPAN
-MASAAKI IWAHORI
-TEL : +81-4-2332-3448
-</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -1367,6 +1360,14 @@
   </si>
   <si>
     <t>{.productName}</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">{customerName}
+{address}
+{receiverName}
+TEL :{telNumber}
+</t>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
@@ -1712,6 +1713,102 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1727,9 +1824,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1738,99 +1832,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2162,441 +2163,458 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A2" s="43" t="s">
-        <v>39</v>
-      </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
+      <c r="A2" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
     </row>
     <row r="3" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="45"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
+      <c r="A3" s="32"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="47"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
+      <c r="A4" s="34"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
     </row>
     <row r="5" spans="1:10" ht="18.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
     </row>
     <row r="6" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="16"/>
-      <c r="J6" s="17"/>
+      <c r="H6" s="47" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="48"/>
+      <c r="J6" s="49"/>
     </row>
     <row r="7" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="39"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
       <c r="G7" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H7" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="I7" s="16"/>
-      <c r="J7" s="17"/>
+        <v>3</v>
+      </c>
+      <c r="H7" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="48"/>
+      <c r="J7" s="49"/>
     </row>
     <row r="8" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="41"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
       <c r="G8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H8" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="I8" s="16"/>
-      <c r="J8" s="17"/>
+        <v>4</v>
+      </c>
+      <c r="H8" s="47" t="s">
+        <v>41</v>
+      </c>
+      <c r="I8" s="48"/>
+      <c r="J8" s="49"/>
     </row>
     <row r="9" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="46"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H9" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" s="16"/>
-      <c r="J9" s="17"/>
+      <c r="H9" s="47" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="48"/>
+      <c r="J9" s="49"/>
     </row>
     <row r="10" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="19"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
+      <c r="A10" s="50"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="51"/>
+      <c r="D10" s="51"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="51"/>
       <c r="G10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="H10" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="I10" s="16"/>
-      <c r="J10" s="17"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="49"/>
     </row>
     <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="G11" s="52"/>
+      <c r="H11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="21"/>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="C12" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>45</v>
-      </c>
       <c r="D12" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E12" s="5"/>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="44"/>
+      <c r="H12" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="G12" s="18"/>
-      <c r="H12" s="6" t="s">
+      <c r="I12" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="J12" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="42"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="42"/>
+      <c r="H13" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I13" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>20</v>
-      </c>
       <c r="J13" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="25"/>
+      <c r="A14" s="41" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="42"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="42"/>
+      <c r="I14" s="43"/>
       <c r="J14" s="11"/>
     </row>
     <row r="15" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="25"/>
+      <c r="A15" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="43"/>
       <c r="J15" s="11"/>
     </row>
     <row r="16" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="25"/>
+      <c r="A16" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="42"/>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="43"/>
       <c r="J16" s="11"/>
     </row>
     <row r="17" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="25"/>
+      <c r="A17" s="41" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="42"/>
+      <c r="F17" s="42"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="42"/>
+      <c r="I17" s="43"/>
       <c r="J17" s="11"/>
     </row>
     <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="36"/>
+      <c r="C18" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="49"/>
-      <c r="C18" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="37"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="37"/>
+      <c r="J18" s="37"/>
     </row>
     <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="49" t="s">
+      <c r="A19" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="36"/>
+      <c r="C19" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="49"/>
-      <c r="C19" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="37"/>
+      <c r="J19" s="37"/>
     </row>
     <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="49" t="s">
+      <c r="A20" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="36"/>
+      <c r="C20" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="49"/>
-      <c r="C20" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
     </row>
     <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="49" t="s">
+      <c r="A21" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="36"/>
+      <c r="C21" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="49"/>
-      <c r="C21" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
     </row>
     <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="49" t="s">
+      <c r="A22" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="36"/>
+      <c r="C22" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="49"/>
-      <c r="C22" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="37"/>
+      <c r="J22" s="37"/>
     </row>
     <row r="23" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="50"/>
-      <c r="C23" s="51" t="s">
-        <v>38</v>
-      </c>
-      <c r="D23" s="51"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
-      <c r="J23" s="51"/>
+      <c r="A23" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23" s="38"/>
+      <c r="C23" s="39" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
     </row>
     <row r="24" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
-      <c r="H24" s="26"/>
-      <c r="I24" s="26"/>
-      <c r="J24" s="26"/>
+      <c r="A24" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
     </row>
     <row r="25" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="29"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="30"/>
+      <c r="A25" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="17"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="31"/>
-      <c r="B26" s="32"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
-      <c r="F26" s="32"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
-      <c r="J26" s="33"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="20"/>
     </row>
     <row r="27" spans="1:10" ht="23.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="34"/>
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="36"/>
+      <c r="A27" s="21"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C20:J20"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:I17"/>
     <mergeCell ref="A24:J24"/>
     <mergeCell ref="G1:J5"/>
     <mergeCell ref="A25:J27"/>
@@ -2613,23 +2631,6 @@
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="C19:J19"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="C20:J20"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A14:I14"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="H8:J8"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.27500000000000002" right="0.118055555555556" top="0.156944444444444" bottom="0.118055555555556" header="0.196527777777778" footer="0.156944444444444"/>

</xml_diff>

<commit_message>
Lambda SCM 2023-10-23 采购价目变更bug 修复
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/PIDomestic.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/PIDomestic.xlsx
@@ -1363,11 +1363,10 @@
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">{customerName}
+    <t>{customerName}
 {address}
 {receiverName}
-TEL :{telNumber}
-</t>
+TEL :{telNumber}</t>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
@@ -1713,6 +1712,45 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1785,9 +1823,6 @@
     <xf numFmtId="179" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1796,42 +1831,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2163,156 +2162,156 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="14" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
     </row>
     <row r="3" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="32"/>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
+      <c r="A3" s="45"/>
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="34"/>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
+      <c r="A4" s="47"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
     </row>
     <row r="5" spans="1:10" ht="18.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
     </row>
     <row r="6" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
       <c r="G6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H6" s="47" t="s">
+      <c r="H6" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="I6" s="48"/>
-      <c r="J6" s="49"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="17"/>
     </row>
     <row r="7" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="26"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
       <c r="G7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H7" s="47" t="s">
+      <c r="H7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="49"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="17"/>
     </row>
     <row r="8" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="28"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
+      <c r="A8" s="41"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
       <c r="G8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H8" s="47" t="s">
+      <c r="H8" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="I8" s="48"/>
-      <c r="J8" s="49"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="17"/>
     </row>
     <row r="9" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="45" t="s">
+      <c r="A9" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="46"/>
-      <c r="C9" s="46"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="46"/>
-      <c r="F9" s="46"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
       <c r="G9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H9" s="47" t="s">
+      <c r="H9" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="I9" s="48"/>
-      <c r="J9" s="49"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="17"/>
     </row>
     <row r="10" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="50"/>
-      <c r="B10" s="51"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
+      <c r="A10" s="19"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
       <c r="G10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H10" s="47" t="s">
+      <c r="H10" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="I10" s="48"/>
-      <c r="J10" s="49"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="17"/>
     </row>
     <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
@@ -2330,10 +2329,10 @@
       <c r="E11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="52" t="s">
+      <c r="F11" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="52"/>
+      <c r="G11" s="21"/>
       <c r="H11" s="2" t="s">
         <v>15</v>
       </c>
@@ -2358,10 +2357,10 @@
         <v>53</v>
       </c>
       <c r="E12" s="5"/>
-      <c r="F12" s="44" t="s">
+      <c r="F12" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="G12" s="44"/>
+      <c r="G12" s="18"/>
       <c r="H12" s="6" t="s">
         <v>47</v>
       </c>
@@ -2373,15 +2372,15 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="41" t="s">
+      <c r="A13" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
       <c r="H13" s="7" t="s">
         <v>50</v>
       </c>
@@ -2393,228 +2392,211 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="41" t="s">
+      <c r="A14" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="43"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="25"/>
       <c r="J14" s="11"/>
     </row>
     <row r="15" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="41" t="s">
+      <c r="A15" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="42"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="43"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="25"/>
       <c r="J15" s="11"/>
     </row>
     <row r="16" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="41" t="s">
+      <c r="A16" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="43"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="25"/>
       <c r="J16" s="11"/>
     </row>
     <row r="17" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="41" t="s">
+      <c r="A17" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="42"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="43"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="25"/>
       <c r="J17" s="11"/>
     </row>
     <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="36"/>
-      <c r="C18" s="37" t="s">
+      <c r="B18" s="49"/>
+      <c r="C18" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37"/>
-      <c r="J18" s="37"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
     </row>
     <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="36"/>
-      <c r="C19" s="40" t="s">
+      <c r="B19" s="49"/>
+      <c r="C19" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="37"/>
-      <c r="J19" s="37"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
     </row>
     <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="37" t="s">
+      <c r="B20" s="49"/>
+      <c r="C20" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="37"/>
-      <c r="I20" s="37"/>
-      <c r="J20" s="37"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
     </row>
     <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="37" t="s">
+      <c r="B21" s="49"/>
+      <c r="C21" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="37"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="37"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
     </row>
     <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="36" t="s">
+      <c r="A22" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="36"/>
-      <c r="C22" s="37" t="s">
+      <c r="B22" s="49"/>
+      <c r="C22" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="37"/>
-      <c r="I22" s="37"/>
-      <c r="J22" s="37"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
     </row>
     <row r="23" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="38"/>
-      <c r="C23" s="39" t="s">
+      <c r="B23" s="50"/>
+      <c r="C23" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="39"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="51"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="51"/>
+      <c r="H23" s="51"/>
+      <c r="I23" s="51"/>
+      <c r="J23" s="51"/>
     </row>
     <row r="24" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
     </row>
     <row r="25" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="17"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="29"/>
+      <c r="J25" s="30"/>
     </row>
     <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="18"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="20"/>
+      <c r="A26" s="31"/>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="33"/>
     </row>
     <row r="27" spans="1:10" ht="23.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="21"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="23"/>
+      <c r="A27" s="34"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="35"/>
+      <c r="I27" s="35"/>
+      <c r="J27" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C20:J20"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A14:I14"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A17:I17"/>
     <mergeCell ref="A24:J24"/>
     <mergeCell ref="G1:J5"/>
     <mergeCell ref="A25:J27"/>
@@ -2631,6 +2613,23 @@
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="C19:J19"/>
     <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C20:J20"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H8:J8"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.27500000000000002" right="0.118055555555556" top="0.156944444444444" bottom="0.118055555555556" header="0.196527777777778" footer="0.156944444444444"/>

</xml_diff>

<commit_message>
Lambda  2023-10-25 迭代ERP-8129 bug 修復
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-oms/src/main/resources/excel/PIDomestic.xlsx
+++ b/erp-server/erp-server-oms/src/main/resources/excel/PIDomestic.xlsx
@@ -297,7 +297,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <r>
       <rPr>
@@ -1289,10 +1289,6 @@
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
   <si>
-    <t>{.materials}</t>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
     <t>{.qty}</t>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
@@ -1367,6 +1363,14 @@
 {address}
 {receiverName}
 TEL :{telNumber}</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.materials}</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>{.imageUrl}</t>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
 </sst>
@@ -1672,7 +1676,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1785,40 +1789,31 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" shrinkToFit="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="179" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
@@ -2171,45 +2166,45 @@
       <c r="E1" s="14"/>
       <c r="F1" s="14"/>
       <c r="G1" s="27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H1" s="27"/>
       <c r="I1" s="27"/>
       <c r="J1" s="27"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="39"/>
       <c r="G2" s="27"/>
       <c r="H2" s="27"/>
       <c r="I2" s="27"/>
       <c r="J2" s="27"/>
     </row>
     <row r="3" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="45"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
+      <c r="A3" s="40"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="42"/>
       <c r="G3" s="27"/>
       <c r="H3" s="27"/>
       <c r="I3" s="27"/>
       <c r="J3" s="27"/>
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="47"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="45"/>
       <c r="G4" s="27"/>
       <c r="H4" s="27"/>
       <c r="I4" s="27"/>
@@ -2231,13 +2226,13 @@
     </row>
     <row r="6" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="38"/>
       <c r="C6" s="38"/>
       <c r="D6" s="38"/>
       <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
+      <c r="F6" s="39"/>
       <c r="G6" s="2" t="s">
         <v>2</v>
       </c>
@@ -2248,12 +2243,12 @@
       <c r="J6" s="17"/>
     </row>
     <row r="7" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="39"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
+      <c r="A7" s="40"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="42"/>
       <c r="G7" s="2" t="s">
         <v>3</v>
       </c>
@@ -2264,12 +2259,12 @@
       <c r="J7" s="17"/>
     </row>
     <row r="8" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="41"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
+      <c r="A8" s="43"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="45"/>
       <c r="G8" s="2" t="s">
         <v>4</v>
       </c>
@@ -2354,21 +2349,23 @@
         <v>44</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E12" s="5"/>
+        <v>52</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="F12" s="18" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G12" s="18"/>
       <c r="H12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J12" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
@@ -2382,13 +2379,13 @@
       <c r="F13" s="24"/>
       <c r="G13" s="24"/>
       <c r="H13" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>19</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.15">
@@ -2448,10 +2445,10 @@
       <c r="J17" s="11"/>
     </row>
     <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="49"/>
+      <c r="B18" s="46"/>
       <c r="C18" s="22" t="s">
         <v>25</v>
       </c>
@@ -2464,11 +2461,11 @@
       <c r="J18" s="22"/>
     </row>
     <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="49" t="s">
+      <c r="A19" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="49"/>
-      <c r="C19" s="52" t="s">
+      <c r="B19" s="46"/>
+      <c r="C19" s="49" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="22"/>
@@ -2480,10 +2477,10 @@
       <c r="J19" s="22"/>
     </row>
     <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="49" t="s">
+      <c r="A20" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="49"/>
+      <c r="B20" s="46"/>
       <c r="C20" s="22" t="s">
         <v>29</v>
       </c>
@@ -2496,10 +2493,10 @@
       <c r="J20" s="22"/>
     </row>
     <row r="21" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="49" t="s">
+      <c r="A21" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="49"/>
+      <c r="B21" s="46"/>
       <c r="C21" s="22" t="s">
         <v>31</v>
       </c>
@@ -2512,10 +2509,10 @@
       <c r="J21" s="22"/>
     </row>
     <row r="22" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="49" t="s">
+      <c r="A22" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="49"/>
+      <c r="B22" s="46"/>
       <c r="C22" s="22" t="s">
         <v>33</v>
       </c>
@@ -2528,20 +2525,20 @@
       <c r="J22" s="22"/>
     </row>
     <row r="23" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="50" t="s">
+      <c r="A23" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="50"/>
-      <c r="C23" s="51" t="s">
+      <c r="B23" s="47"/>
+      <c r="C23" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="51"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="51"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="51"/>
-      <c r="I23" s="51"/>
-      <c r="J23" s="51"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
     </row>
     <row r="24" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="26" t="s">

</xml_diff>